<commit_message>
Migrate news article pages
Automated migration updates generated by Experience Modernization Agent.

Changed files: 59
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-guide-with-page-nav.report.xlsx
+++ b/tools/importer/reports/import-guide-with-page-nav.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="338">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","search-banner","cards-audience","columns-links","columns-campaign","columns-story","cards-news","cards-resources"]</t>
+    <t>["hero","search-banner","cards-audience","list","columns-campaign","columns-story","cards-news","cards-resources"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-05T23:48:01.319Z</t>
+    <t>2026-10-21T01:44:42.721Z</t>
   </si>
   <si>
     <t>Insurance and Care NSW | icare</t>
@@ -133,7 +133,7 @@
     <t>workers-compensation/employers</t>
   </si>
   <si>
-    <t>2026-10-11T09:44:58.930Z</t>
+    <t>2026-10-20T22:26:56.105Z</t>
   </si>
   <si>
     <t>Employers | icare</t>
@@ -154,7 +154,7 @@
     <t>section-overview-hub</t>
   </si>
   <si>
-    <t>2026-10-13T22:24:07.431Z</t>
+    <t>2026-10-20T22:26:30.758Z</t>
   </si>
   <si>
     <t>Small business hub | icare</t>
@@ -175,7 +175,7 @@
     <t>hero-image-content-with-sidebar</t>
   </si>
   <si>
-    <t>2026-10-13T22:24:20.957Z</t>
+    <t>2026-10-20T22:26:41.952Z</t>
   </si>
   <si>
     <t>Notify us of an injury or make a claim | icare</t>
@@ -184,6 +184,96 @@
     <t>https://www.icare.nsw.gov.au/employers/make-a-claim/notify-us-of-an-injury-or-make-a-claim</t>
   </si>
   <si>
+    <t>news-and-stories/2024/adaptive-sports-helps-jarrod-reimagine-whats-possible.report.json</t>
+  </si>
+  <si>
+    <t>["cards-promo","embed-video","cards-news"]</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/adaptive-sports-helps-jarrod-reimagine-whats-possible</t>
+  </si>
+  <si>
+    <t>news-story-with-video</t>
+  </si>
+  <si>
+    <t>2026-10-21T01:28:41.607Z</t>
+  </si>
+  <si>
+    <t>Adaptive sports helps Jarrod reimagine whats possible | icare</t>
+  </si>
+  <si>
+    <t>https://www.icare.nsw.gov.au/news-and-stories/2024/adaptive-sports-helps-jarrod-reimagine-whats-possible</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/annabelle-shares-her-passion-for-adaptive-sports.report.json</t>
+  </si>
+  <si>
+    <t>["cards-promo","quote-pull","embed-video","cards-news"]</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/annabelle-shares-her-passion-for-adaptive-sports</t>
+  </si>
+  <si>
+    <t>2026-10-21T01:28:50.004Z</t>
+  </si>
+  <si>
+    <t>Annabelle shares her passion for adaptive sports | icare</t>
+  </si>
+  <si>
+    <t>https://www.icare.nsw.gov.au/news-and-stories/2024/annabelle-shares-her-passion-for-adaptive-sports</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/reimagining-your-life.report.json</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/reimagining-your-life</t>
+  </si>
+  <si>
+    <t>2026-10-21T01:29:44.286Z</t>
+  </si>
+  <si>
+    <t>Reimagining your life | icare</t>
+  </si>
+  <si>
+    <t>https://www.icare.nsw.gov.au/news-and-stories/2024/reimagining-your-life</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/shine-magazine-summer-2024-edition-is-out-now.report.json</t>
+  </si>
+  <si>
+    <t>["cards-promo","quote-pull","cards-news"]</t>
+  </si>
+  <si>
+    <t>news-and-stories/2024/shine-magazine-summer-2024-edition-is-out-now</t>
+  </si>
+  <si>
+    <t>2026-10-21T01:29:55.301Z</t>
+  </si>
+  <si>
+    <t>Shine Magazine summer 2024 edition is out now | icare</t>
+  </si>
+  <si>
+    <t>https://www.icare.nsw.gov.au/news-and-stories/2024/shine-magazine-summer-2024-edition-is-out-now</t>
+  </si>
+  <si>
+    <t>news-and-stories/2025/icare-safeguards-nsw-workers-with-new-lung-health-mobile-clinic.report.json</t>
+  </si>
+  <si>
+    <t>["cards-promo","columns","quote-bordered","quote-pull","cards-news"]</t>
+  </si>
+  <si>
+    <t>news-and-stories/2025/icare-safeguards-nsw-workers-with-new-lung-health-mobile-clinic</t>
+  </si>
+  <si>
+    <t>2026-10-21T01:30:07.156Z</t>
+  </si>
+  <si>
+    <t>icare safeguards NSW workers with new Lung Health Mobile Clinic | icare</t>
+  </si>
+  <si>
+    <t>https://www.icare.nsw.gov.au/news-and-stories/2025/icare-safeguards-nsw-workers-with-new-lung-health-mobile-clinic</t>
+  </si>
+  <si>
     <t>workers-compensation/employers/apprentice-incentive-scheme.report.json</t>
   </si>
   <si>
@@ -535,7 +625,7 @@
     <t>workers-compensation/employers/manage-your-policy/renew-your-policy</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:17.501Z</t>
+    <t>2026-10-21T01:45:39.480Z</t>
   </si>
   <si>
     <t>Renew your Workers Insurance policy | icare</t>
@@ -661,7 +751,7 @@
     <t>workers-compensation/employers/new-policy/premium-calculation-experience-rated</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:43.025Z</t>
+    <t>2026-10-21T01:46:40.031Z</t>
   </si>
   <si>
     <t>Premium calculation experience-rated | icare</t>
@@ -775,13 +865,13 @@
     <t>workers-compensation/employers/prevention-and-education/adssi-limited.report.json</t>
   </si>
   <si>
-    <t>["hero","cards-audience","embed-video"]</t>
+    <t>["hero","cards-audience","embed-video","quote-bordered","quote-bordered"]</t>
   </si>
   <si>
     <t>workers-compensation/employers/prevention-and-education/adssi-limited</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:01.925Z</t>
+    <t>2026-10-21T01:46:31.333Z</t>
   </si>
   <si>
     <t>ADSSI Limited | icare</t>
@@ -793,10 +883,13 @@
     <t>workers-compensation/employers/prevention-and-education/asbjv.report.json</t>
   </si>
   <si>
+    <t>["hero","cards-audience","quote-bordered","quote-bordered"]</t>
+  </si>
+  <si>
     <t>workers-compensation/employers/prevention-and-education/asbjv</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:09.269Z</t>
+    <t>2026-10-20T22:22:20.748Z</t>
   </si>
   <si>
     <t>ASBJV | icare</t>
@@ -811,7 +904,7 @@
     <t>workers-compensation/employers/prevention-and-education/ebos-group</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:17.548Z</t>
+    <t>2026-10-20T22:22:29.134Z</t>
   </si>
   <si>
     <t>EBOS Group | icare</t>
@@ -877,7 +970,7 @@
     <t>workers-compensation/employers/prevention-and-education/metcash</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:44.308Z</t>
+    <t>2026-10-20T22:23:22.286Z</t>
   </si>
   <si>
     <t>Metcash | icare</t>
@@ -919,13 +1012,13 @@
     <t>workers-compensation/employers/prevention-and-education/weathertex.report.json</t>
   </si>
   <si>
-    <t>["hero","cards-audience","embed-video","embed-video"]</t>
+    <t>["hero","cards-audience","embed-video","embed-video","quote-bordered","quote-bordered"]</t>
   </si>
   <si>
     <t>workers-compensation/employers/prevention-and-education/weathertex</t>
   </si>
   <si>
-    <t>2026-10-20T04:01:53.447Z</t>
+    <t>2026-10-20T22:24:16.095Z</t>
   </si>
   <si>
     <t>Weathertex | icare</t>
@@ -1320,7 +1413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1698,1065 +1791,1195 @@
         <v>87</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G15" t="s">
-        <v>31</v>
+        <v>92</v>
       </c>
       <c r="H15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G16" t="s">
-        <v>36</v>
+        <v>98</v>
       </c>
       <c r="H16" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" t="s">
         <v>95</v>
       </c>
-      <c r="B17" t="s">
-        <v>96</v>
-      </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="F17" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="G17" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H17" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B18" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F18" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H18" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C19" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G19" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H19" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="H20" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G21" t="s">
-        <v>121</v>
+        <v>36</v>
       </c>
       <c r="H21" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B22" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C22" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="F22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G22" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H22" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>132</v>
       </c>
       <c r="C23" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F23" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G23" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H23" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B24" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C24" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>137</v>
+        <v>90</v>
       </c>
       <c r="F24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G24" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C25" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F25" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G25" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H25" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B26" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="C26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G26" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H26" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>154</v>
       </c>
       <c r="C27" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F27" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G27" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H27" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F28" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G28" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H28" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>165</v>
       </c>
       <c r="C29" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>60</v>
+        <v>167</v>
       </c>
       <c r="F29" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G29" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H29" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B30" t="s">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F30" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="G30" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="H30" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B31" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
       <c r="C31" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F31" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="G31" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H31" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>138</v>
       </c>
       <c r="C32" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F32" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="G32" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="H32" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F33" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="G33" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="H33" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="C34" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F34" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="G34" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="H34" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B35" t="s">
-        <v>193</v>
+        <v>95</v>
       </c>
       <c r="C35" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D35" t="s">
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F35" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="G35" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="H35" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B36" t="s">
-        <v>108</v>
+        <v>177</v>
       </c>
       <c r="C36" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F36" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="G36" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="H36" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="C37" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F37" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="G37" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="H37" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C38" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F38" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="G38" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="H38" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B39" t="s">
-        <v>214</v>
+        <v>138</v>
       </c>
       <c r="C39" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F39" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="G39" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="H39" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C40" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F40" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G40" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H40" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F41" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G41" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="H41" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B42" t="s">
-        <v>231</v>
+        <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F42" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G42" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="H42" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B43" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C43" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F43" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G43" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H43" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B44" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C44" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F44" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G44" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H44" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B45" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C45" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F45" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G45" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H45" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B46" t="s">
-        <v>254</v>
+        <v>106</v>
       </c>
       <c r="C46" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
       </c>
       <c r="E46" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F46" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G46" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H46" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B47" t="s">
-        <v>65</v>
+        <v>261</v>
       </c>
       <c r="C47" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
       </c>
       <c r="E47" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F47" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G47" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="H47" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B48" t="s">
-        <v>254</v>
+        <v>138</v>
       </c>
       <c r="C48" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
       </c>
       <c r="E48" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F48" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G48" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="H48" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B49" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C49" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F49" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G49" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="H49" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B50" t="s">
-        <v>65</v>
+        <v>278</v>
       </c>
       <c r="C50" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
       </c>
       <c r="E50" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F50" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="G50" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="H50" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B51" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C51" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D51" t="s">
         <v>11</v>
       </c>
       <c r="E51" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F51" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="G51" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="H51" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B52" t="s">
-        <v>254</v>
+        <v>290</v>
       </c>
       <c r="C52" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="D52" t="s">
         <v>11</v>
       </c>
       <c r="E52" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G52" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="H52" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B53" t="s">
-        <v>76</v>
+        <v>284</v>
       </c>
       <c r="C53" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D53" t="s">
         <v>11</v>
       </c>
       <c r="E53" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F53" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="G53" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="H53" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B54" t="s">
-        <v>76</v>
+        <v>301</v>
       </c>
       <c r="C54" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="D54" t="s">
         <v>11</v>
       </c>
       <c r="E54" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F54" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="G54" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="H54" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B55" t="s">
-        <v>302</v>
+        <v>95</v>
       </c>
       <c r="C55" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D55" t="s">
         <v>11</v>
       </c>
       <c r="E55" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F55" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G55" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="H55" t="s">
-        <v>306</v>
+        <v>310</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>311</v>
+      </c>
+      <c r="B56" t="s">
+        <v>312</v>
+      </c>
+      <c r="C56" t="s">
+        <v>313</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>90</v>
+      </c>
+      <c r="F56" t="s">
+        <v>314</v>
+      </c>
+      <c r="G56" t="s">
+        <v>315</v>
+      </c>
+      <c r="H56" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>317</v>
+      </c>
+      <c r="B57" t="s">
+        <v>284</v>
+      </c>
+      <c r="C57" t="s">
+        <v>318</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>90</v>
+      </c>
+      <c r="F57" t="s">
+        <v>319</v>
+      </c>
+      <c r="G57" t="s">
+        <v>320</v>
+      </c>
+      <c r="H57" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>322</v>
+      </c>
+      <c r="B58" t="s">
+        <v>106</v>
+      </c>
+      <c r="C58" t="s">
+        <v>323</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>90</v>
+      </c>
+      <c r="F58" t="s">
+        <v>324</v>
+      </c>
+      <c r="G58" t="s">
+        <v>325</v>
+      </c>
+      <c r="H58" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>327</v>
+      </c>
+      <c r="B59" t="s">
+        <v>106</v>
+      </c>
+      <c r="C59" t="s">
+        <v>328</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>90</v>
+      </c>
+      <c r="F59" t="s">
+        <v>329</v>
+      </c>
+      <c r="G59" t="s">
+        <v>330</v>
+      </c>
+      <c r="H59" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>332</v>
+      </c>
+      <c r="B60" t="s">
+        <v>333</v>
+      </c>
+      <c r="C60" t="s">
+        <v>334</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>90</v>
+      </c>
+      <c r="F60" t="s">
+        <v>335</v>
+      </c>
+      <c r="G60" t="s">
+        <v>336</v>
+      </c>
+      <c r="H60" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add embed-video block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 64
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-guide-with-page-nav.report.xlsx
+++ b/tools/importer/reports/import-guide-with-page-nav.report.xlsx
@@ -133,7 +133,7 @@
     <t>workers-compensation/employers</t>
   </si>
   <si>
-    <t>2026-10-20T22:26:56.105Z</t>
+    <t>2026-10-21T01:46:53.801Z</t>
   </si>
   <si>
     <t>Employers | icare</t>
@@ -154,7 +154,7 @@
     <t>section-overview-hub</t>
   </si>
   <si>
-    <t>2026-10-20T22:26:30.758Z</t>
+    <t>2026-10-21T01:47:51.170Z</t>
   </si>
   <si>
     <t>Small business hub | icare</t>
@@ -175,7 +175,7 @@
     <t>hero-image-content-with-sidebar</t>
   </si>
   <si>
-    <t>2026-10-20T22:26:41.952Z</t>
+    <t>2026-10-21T01:48:07.597Z</t>
   </si>
   <si>
     <t>Notify us of an injury or make a claim | icare</t>
@@ -196,7 +196,7 @@
     <t>news-story-with-video</t>
   </si>
   <si>
-    <t>2026-10-21T01:28:41.607Z</t>
+    <t>2026-10-28T09:50:32.547Z</t>
   </si>
   <si>
     <t>Adaptive sports helps Jarrod reimagine whats possible | icare</t>
@@ -214,7 +214,7 @@
     <t>news-and-stories/2024/annabelle-shares-her-passion-for-adaptive-sports</t>
   </si>
   <si>
-    <t>2026-10-21T01:28:50.004Z</t>
+    <t>2026-10-28T09:51:25.119Z</t>
   </si>
   <si>
     <t>Annabelle shares her passion for adaptive sports | icare</t>
@@ -229,7 +229,7 @@
     <t>news-and-stories/2024/reimagining-your-life</t>
   </si>
   <si>
-    <t>2026-10-21T01:29:44.286Z</t>
+    <t>2026-10-28T09:51:33.673Z</t>
   </si>
   <si>
     <t>Reimagining your life | icare</t>
@@ -247,7 +247,7 @@
     <t>news-and-stories/2024/shine-magazine-summer-2024-edition-is-out-now</t>
   </si>
   <si>
-    <t>2026-10-21T01:29:55.301Z</t>
+    <t>2026-10-28T09:51:45.589Z</t>
   </si>
   <si>
     <t>Shine Magazine summer 2024 edition is out now | icare</t>
@@ -265,7 +265,7 @@
     <t>news-and-stories/2025/icare-safeguards-nsw-workers-with-new-lung-health-mobile-clinic</t>
   </si>
   <si>
-    <t>2026-10-21T01:30:07.156Z</t>
+    <t>2026-10-28T09:51:53.846Z</t>
   </si>
   <si>
     <t>icare safeguards NSW workers with new Lung Health Mobile Clinic | icare</t>
@@ -286,7 +286,7 @@
     <t>guide-with-page-nav</t>
   </si>
   <si>
-    <t>2026-10-20T03:54:50.094Z</t>
+    <t>2026-10-28T10:15:08.989Z</t>
   </si>
   <si>
     <t>Apprentice Incentive Scheme | icare</t>
@@ -304,7 +304,7 @@
     <t>workers-compensation/employers/classifying-your-workers</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:00.589Z</t>
+    <t>2026-10-28T10:15:17.307Z</t>
   </si>
   <si>
     <t>Classifying Workers or Contractors for Workers Compensation | icare</t>
@@ -319,7 +319,7 @@
     <t>workers-compensation/employers/forms-and-resources</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:08.559Z</t>
+    <t>2026-10-28T10:15:28.071Z</t>
   </si>
   <si>
     <t>Forms and resources | icare</t>
@@ -337,7 +337,7 @@
     <t>workers-compensation/employers/how-much-will-it-cost</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:17.699Z</t>
+    <t>2026-10-28T10:15:36.212Z</t>
   </si>
   <si>
     <t>Costs and premiums | icare</t>
@@ -355,7 +355,7 @@
     <t>workers-compensation/employers/insurance-for-related-businesses</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:26.791Z</t>
+    <t>2026-10-28T10:15:45.768Z</t>
   </si>
   <si>
     <t>What is Grouping Insurance for Related Businesses? | icare</t>
@@ -415,7 +415,7 @@
     <t>workers-compensation/employers/understanding-icare-and-workers-compensation</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:04.735Z</t>
+    <t>2026-10-28T10:24:09.532Z</t>
   </si>
   <si>
     <t>Understanding ​​icare and Workers Compensation | icare</t>
@@ -433,7 +433,7 @@
     <t>workers-compensation/employers/whats-covered</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:15.887Z</t>
+    <t>2026-10-28T10:24:17.285Z</t>
   </si>
   <si>
     <t>Whats covered | icare</t>
@@ -448,7 +448,7 @@
     <t>workers-compensation/employers/whats-new</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:24.946Z</t>
+    <t>2026-10-28T10:24:25.656Z</t>
   </si>
   <si>
     <t>What's new in Workers Compensation | icare</t>
@@ -463,7 +463,7 @@
     <t>workers-compensation/employers/who-needs-a-policy</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:36.687Z</t>
+    <t>2026-10-28T10:24:38.662Z</t>
   </si>
   <si>
     <t>Who needs a policy | icare</t>
@@ -481,7 +481,7 @@
     <t>workers-compensation/employers/workers-compensation-reform-faqs</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:44.393Z</t>
+    <t>2026-10-28T10:24:48.165Z</t>
   </si>
   <si>
     <t>Workers Compensation Reform FAQs | icare</t>
@@ -496,7 +496,7 @@
     <t>workers-compensation/employers/your-responsibilities-as-an-employer</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:51.736Z</t>
+    <t>2026-10-28T10:24:56.712Z</t>
   </si>
   <si>
     <t>Your responsibilities | icare</t>
@@ -532,7 +532,7 @@
     <t>workers-compensation/employers/manage-your-policy/cancel-your-workers-insurance-policy</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:39.086Z</t>
+    <t>2026-10-28T10:15:57.349Z</t>
   </si>
   <si>
     <t>Cancel your workers insurance policy | icare</t>
@@ -550,7 +550,7 @@
     <t>workers-compensation/employers/manage-your-policy/declaring-wages</t>
   </si>
   <si>
-    <t>2026-10-20T03:54:39.837Z</t>
+    <t>2026-10-28T10:14:58.989Z</t>
   </si>
   <si>
     <t>Declaring Wages to Calculate Workers Compensation premiums | icare</t>
@@ -565,7 +565,7 @@
     <t>workers-compensation/employers/manage-your-policy/download-a-certificate-of-currency</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:50.169Z</t>
+    <t>2026-10-28T10:16:04.939Z</t>
   </si>
   <si>
     <t>Download a Certificate of Currency | icare</t>
@@ -580,7 +580,7 @@
     <t>workers-compensation/employers/manage-your-policy/faqs-wage-audit-process</t>
   </si>
   <si>
-    <t>2026-10-20T03:56:03.695Z</t>
+    <t>2026-10-28T10:16:16.504Z</t>
   </si>
   <si>
     <t>FAQs Wage Audit Process | icare</t>
@@ -595,7 +595,7 @@
     <t>workers-compensation/employers/manage-your-policy/how-to-access-your-monthly-cost-of-claims-report</t>
   </si>
   <si>
-    <t>2026-10-20T03:56:10.422Z</t>
+    <t>2026-10-28T10:16:29.612Z</t>
   </si>
   <si>
     <t>How to access your monthly Cost of Claims report | icare</t>
@@ -610,7 +610,7 @@
     <t>workers-compensation/employers/manage-your-policy/premium-disputes</t>
   </si>
   <si>
-    <t>2026-10-20T03:56:22.400Z</t>
+    <t>2026-10-28T10:16:39.069Z</t>
   </si>
   <si>
     <t>Premium disputes | icare</t>
@@ -625,7 +625,7 @@
     <t>workers-compensation/employers/manage-your-policy/renew-your-policy</t>
   </si>
   <si>
-    <t>2026-10-21T01:45:39.480Z</t>
+    <t>2026-10-28T10:17:32.428Z</t>
   </si>
   <si>
     <t>Renew your Workers Insurance policy | icare</t>
@@ -640,7 +640,7 @@
     <t>workers-compensation/employers/manage-your-policy/update-your-policy-details</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:28.007Z</t>
+    <t>2026-10-28T10:17:45.308Z</t>
   </si>
   <si>
     <t>Update your policy details | icare</t>
@@ -655,7 +655,7 @@
     <t>workers-compensation/employers/new-policy/2026-premium-rate-freeze</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:41.380Z</t>
+    <t>2026-10-28T10:17:57.660Z</t>
   </si>
   <si>
     <t>2026 Premium Rate Freeze | icare</t>
@@ -670,7 +670,7 @@
     <t>workers-compensation/employers/new-policy/claims-performance-adjustment-rates</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:52.559Z</t>
+    <t>2026-10-28T10:18:09.118Z</t>
   </si>
   <si>
     <t>Claims performance adjustment rates | icare</t>
@@ -688,7 +688,7 @@
     <t>workers-compensation/employers/new-policy/how-to-lower-your-premium</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:02.333Z</t>
+    <t>2026-10-28T10:18:19.429Z</t>
   </si>
   <si>
     <t>How to lower your premium | icare</t>
@@ -703,7 +703,7 @@
     <t>workers-compensation/employers/new-policy/how-to-pay-your-premium</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:10.843Z</t>
+    <t>2026-10-28T10:18:32.284Z</t>
   </si>
   <si>
     <t>How to pay your premium | icare</t>
@@ -718,7 +718,7 @@
     <t>workers-compensation/employers/new-policy/loss-prevention-and-recovery</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:18.715Z</t>
+    <t>2026-10-28T10:18:41.251Z</t>
   </si>
   <si>
     <t>Loss Prevention and Recovery Products for Calculating Premium | icare</t>
@@ -733,7 +733,7 @@
     <t>workers-compensation/employers/new-policy/multiple-business-activities-and-wic-classification</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:30.386Z</t>
+    <t>2026-10-28T10:18:54.391Z</t>
   </si>
   <si>
     <t>Multiple business activities and WIC classification | icare</t>
@@ -751,7 +751,7 @@
     <t>workers-compensation/employers/new-policy/premium-calculation-experience-rated</t>
   </si>
   <si>
-    <t>2026-10-21T01:46:40.031Z</t>
+    <t>2026-10-28T10:19:06.023Z</t>
   </si>
   <si>
     <t>Premium calculation experience-rated | icare</t>
@@ -769,7 +769,7 @@
     <t>workers-compensation/employers/new-policy/premium-calculation-for-small-employers</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:55.911Z</t>
+    <t>2026-10-28T10:19:18.644Z</t>
   </si>
   <si>
     <t>Premium calculation for small employers | icare</t>
@@ -784,7 +784,7 @@
     <t>workers-compensation/employers/new-policy/take-out-a-policy</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:07.318Z</t>
+    <t>2026-10-28T10:19:39.345Z</t>
   </si>
   <si>
     <t>Take out a policy | icare</t>
@@ -802,7 +802,7 @@
     <t>workers-compensation/employers/new-policy/understanding-wics-and-premium-rates</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:19.064Z</t>
+    <t>2026-10-28T10:19:51.263Z</t>
   </si>
   <si>
     <t>Understanding WICS and premium rates | icare</t>
@@ -817,7 +817,7 @@
     <t>workers-compensation/employers/new-policy/understanding-your-cover</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:31.385Z</t>
+    <t>2026-10-28T10:20:03.027Z</t>
   </si>
   <si>
     <t>Understanding your cover | icare</t>
@@ -835,7 +835,7 @@
     <t>workers-compensation/employers/new-policy/understanding-your-premium</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:42.489Z</t>
+    <t>2026-10-28T10:20:14.827Z</t>
   </si>
   <si>
     <t>Understanding your premium | icare</t>
@@ -853,7 +853,7 @@
     <t>workers-compensation/employers/new-policy/what-is-premium-capping-and-how-does-it-work</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:53.640Z</t>
+    <t>2026-10-28T10:20:24.496Z</t>
   </si>
   <si>
     <t>What is premium capping and how does it work? | icare</t>
@@ -871,7 +871,7 @@
     <t>workers-compensation/employers/prevention-and-education/adssi-limited</t>
   </si>
   <si>
-    <t>2026-10-21T01:46:31.333Z</t>
+    <t>2026-10-28T10:20:34.243Z</t>
   </si>
   <si>
     <t>ADSSI Limited | icare</t>
@@ -889,7 +889,7 @@
     <t>workers-compensation/employers/prevention-and-education/asbjv</t>
   </si>
   <si>
-    <t>2026-10-20T22:22:20.748Z</t>
+    <t>2026-10-28T10:20:42.143Z</t>
   </si>
   <si>
     <t>ASBJV | icare</t>
@@ -904,7 +904,7 @@
     <t>workers-compensation/employers/prevention-and-education/ebos-group</t>
   </si>
   <si>
-    <t>2026-10-20T22:22:29.134Z</t>
+    <t>2026-10-28T10:21:35.670Z</t>
   </si>
   <si>
     <t>EBOS Group | icare</t>
@@ -922,7 +922,7 @@
     <t>workers-compensation/employers/prevention-and-education/expert-consultation</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:25.683Z</t>
+    <t>2026-10-28T10:21:43.977Z</t>
   </si>
   <si>
     <t>Expert consultation | icare</t>
@@ -937,7 +937,7 @@
     <t>workers-compensation/employers/prevention-and-education/injury-prevention-resource-hub</t>
   </si>
   <si>
-    <t>2026-10-20T04:03:03.005Z</t>
+    <t>2026-10-28T10:25:04.443Z</t>
   </si>
   <si>
     <t>Injury prevention resource hub | icare</t>
@@ -955,7 +955,7 @@
     <t>workers-compensation/employers/prevention-and-education/injury-prevention</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:35.785Z</t>
+    <t>2026-10-28T10:21:54.242Z</t>
   </si>
   <si>
     <t>Injury Prevention | icare</t>
@@ -970,7 +970,7 @@
     <t>workers-compensation/employers/prevention-and-education/metcash</t>
   </si>
   <si>
-    <t>2026-10-20T22:23:22.286Z</t>
+    <t>2026-10-28T10:22:47.893Z</t>
   </si>
   <si>
     <t>Metcash | icare</t>
@@ -985,7 +985,7 @@
     <t>workers-compensation/employers/prevention-and-education/the-safety-locker</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:52.169Z</t>
+    <t>2026-10-28T10:22:55.542Z</t>
   </si>
   <si>
     <t>The safety locker | icare</t>
@@ -1000,7 +1000,7 @@
     <t>workers-compensation/employers/prevention-and-education/training-programs</t>
   </si>
   <si>
-    <t>2026-10-20T04:01:01.339Z</t>
+    <t>2026-10-28T10:23:02.915Z</t>
   </si>
   <si>
     <t>Training programs | icare</t>
@@ -1018,7 +1018,7 @@
     <t>workers-compensation/employers/prevention-and-education/weathertex</t>
   </si>
   <si>
-    <t>2026-10-20T22:24:16.095Z</t>
+    <t>2026-10-28T10:23:55.650Z</t>
   </si>
   <si>
     <t>Weathertex | icare</t>

</xml_diff>